<commit_message>
changed carlota's user permission to USER for testing
</commit_message>
<xml_diff>
--- a/RevitMappingData/ProjectRoleDatabase.xlsx
+++ b/RevitMappingData/ProjectRoleDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZAMORAMARIACARLOTAGA\Documents\GitHub\pocDataRepo\RevitMappingData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F48EE0B5-2EA4-4D04-8C96-C534398F55C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECF9488-13A9-4328-ABAB-5DBD7BB46860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20085" yWindow="-15135" windowWidth="21510" windowHeight="11235" xr2:uid="{D777F439-9358-4388-BAEA-A8A675FE2155}"/>
   </bookViews>
@@ -553,7 +553,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Carlota's role changed back to Admin
</commit_message>
<xml_diff>
--- a/RevitMappingData/ProjectRoleDatabase.xlsx
+++ b/RevitMappingData/ProjectRoleDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZAMORAMARIACARLOTAGA\Documents\GitHub\pocDataRepo\RevitMappingData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECF9488-13A9-4328-ABAB-5DBD7BB46860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47972E6F-E698-4CB7-8A69-11173CDC4588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20085" yWindow="-15135" windowWidth="21510" windowHeight="11235" xr2:uid="{D777F439-9358-4388-BAEA-A8A675FE2155}"/>
   </bookViews>
@@ -553,7 +553,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>

</xml_diff>